<commit_message>
Add clean database rebuild script with updated standards and modules data.
- Add rebuild_correlation_database.py: Complete database rebuild script for correlation data
- Add updated modules matrix with clean grade/subject separation
- Fix standards data: add MS-PS4-3, fix MS-ESS2-2 typo, remove invalid MS-LS3-3
- Remove outdated NGSS standards markdown file
- Script supports both local SQLite and Render PostgreSQL with backup option
- Maintains data integrity and preserves non-correlation data (users, drafts, etc.)

🤖 Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/standards/CC and NGSS Standards.xlsx
+++ b/data/standards/CC and NGSS Standards.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="4030" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BF6F956-11A1-45B1-BF91-AA4435C5C03F}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moriahplacer/Desktop/Mo's Vault/nola.docs/data/standards/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FBD920-2526-9941-AF37-B099BE8FDCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30420" yWindow="-2180" windowWidth="20180" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MS Science " sheetId="13" r:id="rId1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="435">
   <si>
     <t>NGSS</t>
   </si>
@@ -323,9 +328,6 @@
   </si>
   <si>
     <t>Develop a model to describe the cycling of Earth’s materials and the flow of energy that drives this process.</t>
-  </si>
-  <si>
-    <t>MSS-ESS2-2</t>
   </si>
   <si>
     <t xml:space="preserve">Construct an explanation based on evidence for how geoscience processes have changed Earth’s surface at varying time and spatial scales. </t>
@@ -976,7 +978,7 @@
         <sz val="8"/>
         <color theme="1"/>
         <rFont val="Courier New"/>
-        <charset val="1"/>
+        <family val="1"/>
       </rPr>
       <t>.</t>
     </r>
@@ -1035,7 +1037,7 @@
         <sz val="6"/>
         <color theme="1"/>
         <rFont val="Arial"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t>2</t>
     </r>
@@ -1044,7 +1046,7 @@
         <sz val="9"/>
         <color theme="1"/>
         <rFont val="Arial"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t>= qthat has the same solutions. Derive the quadratic formula from this form.</t>
     </r>
@@ -1061,7 +1063,7 @@
         <sz val="6"/>
         <color theme="1"/>
         <rFont val="Arial"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t>2</t>
     </r>
@@ -1070,7 +1072,7 @@
         <sz val="9"/>
         <color theme="1"/>
         <rFont val="Arial"/>
-        <charset val="1"/>
+        <family val="2"/>
       </rPr>
       <t>= 49), taking square roots, completing the square, the quadratic formula,and factoring, as appropriate to the initial form of the equation. Recognize when the quadratic formula gives complex solutions and write them as "no real solution.”</t>
     </r>
@@ -1404,13 +1406,22 @@
   </si>
   <si>
     <t>Use a computer simulation to model the impact of proposed solutions to a complex real-world problem with numerous criteria and constraints on interactions within and between systems relevant to the problem.</t>
+  </si>
+  <si>
+    <t>MS-PS4-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrate qualitative scientific and technical information to support the claim that digitized signals are a more reliable way to encode and transmit information than analog signals. </t>
+  </si>
+  <si>
+    <t>MS-ESS2-2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1437,68 +1448,74 @@
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="6"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Courier New"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF333333"/>
       <name val="Helvetica Neue"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1601,9 +1618,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1641,7 +1658,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1747,7 +1764,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1889,7 +1906,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1897,14 +1914,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A257809-108C-4F20-8BE1-397D7319946A}">
-  <dimension ref="A1:B59"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="91.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="91.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1912,7 +1929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="30.75">
+    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
@@ -1920,7 +1937,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="30.75">
+    <row r="3" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -1928,7 +1945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30.75">
+    <row r="4" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
@@ -1936,7 +1953,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="30.75">
+    <row r="5" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
@@ -1944,7 +1961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30.75">
+    <row r="6" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1952,7 +1969,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30.75">
+    <row r="7" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>12</v>
       </c>
@@ -1960,7 +1977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="45.75">
+    <row r="8" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
@@ -1968,7 +1985,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="45.75">
+    <row r="9" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>16</v>
       </c>
@@ -1976,7 +1993,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="76.5">
+    <row r="10" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
@@ -1984,7 +2001,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45.75">
+    <row r="11" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
@@ -1992,7 +2009,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45.75">
+    <row r="12" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
@@ -2000,7 +2017,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="45.75">
+    <row r="13" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>24</v>
       </c>
@@ -2008,7 +2025,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="45.75">
+    <row r="14" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>26</v>
       </c>
@@ -2016,7 +2033,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="30.75">
+    <row r="15" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>28</v>
       </c>
@@ -2024,7 +2041,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="45.75">
+    <row r="16" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>30</v>
       </c>
@@ -2032,7 +2049,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="30.75">
+    <row r="17" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>32</v>
       </c>
@@ -2040,7 +2057,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="60.75">
+    <row r="18" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>34</v>
       </c>
@@ -2048,7 +2065,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="45.75">
+    <row r="19" spans="1:2" ht="48" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>36</v>
       </c>
@@ -2056,324 +2073,332 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="45.75">
+    <row r="20" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B21" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="45.75">
-      <c r="A21" s="6" t="s">
+    <row r="22" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B22" s="10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="30.75">
-      <c r="A22" s="6" t="s">
+    <row r="23" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B23" s="10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="45.75">
-      <c r="A23" s="6" t="s">
+    <row r="24" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B24" s="10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="30.75">
-      <c r="A24" s="6" t="s">
+    <row r="25" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B25" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="30.75">
-      <c r="A25" s="6" t="s">
+    <row r="26" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B26" s="10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="30.75">
-      <c r="A26" s="6" t="s">
+    <row r="27" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B27" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="33.75">
-      <c r="A27" s="6" t="s">
+    <row r="28" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B28" s="16" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="45.75">
-      <c r="A28" s="6" t="s">
+    <row r="29" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B29" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="45.75">
-      <c r="A29" s="6" t="s">
+    <row r="30" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B30" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="45.75">
-      <c r="A30" s="6" t="s">
+    <row r="31" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B31" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="30.75">
-      <c r="A31" s="6" t="s">
+    <row r="32" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B32" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
-      <c r="A32" s="6" t="s">
+    <row r="33" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B33" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="45.75">
-      <c r="A33" s="6" t="s">
+    <row r="34" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B34" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="30.75">
-      <c r="A34" s="6" t="s">
+    <row r="35" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B35" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="45.75">
-      <c r="A35" s="6" t="s">
+    <row r="36" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B36" s="10" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="30.75">
-      <c r="A36" s="6" t="s">
+    <row r="37" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B37" s="10" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="30.75">
-      <c r="A37" s="6" t="s">
+    <row r="38" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B38" s="10" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="45.75">
-      <c r="A38" s="6" t="s">
+    <row r="39" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B39" s="10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="30.75">
-      <c r="A39" s="6" t="s">
+    <row r="40" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B40" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="30.75">
-      <c r="A40" s="6" t="s">
+    <row r="41" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B41" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="45.75">
-      <c r="A41" s="6" t="s">
+    <row r="42" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="10" t="s">
+      <c r="B42" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="30.75">
-      <c r="A42" s="6" t="s">
+    <row r="43" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B43" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="30.75">
-      <c r="A43" s="6" t="s">
+    <row r="44" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B44" s="10" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="30.75">
-      <c r="A44" s="6" t="s">
+    <row r="45" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B45" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="30.75">
-      <c r="A45" s="6" t="s">
+    <row r="46" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B45" s="10" t="s">
+      <c r="B46" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="30.75">
-      <c r="A46" s="6" t="s">
+    <row r="47" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A47" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="B47" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="10" t="s">
+    </row>
+    <row r="48" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" ht="30.75">
-      <c r="A47" s="6" t="s">
+      <c r="B48" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="10" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A49" s="6" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" ht="30.75">
-      <c r="A48" s="6" t="s">
+      <c r="B49" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="10" t="s">
+    </row>
+    <row r="50" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="30.75">
-      <c r="A49" s="6" t="s">
+      <c r="B50" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="B49" s="10" t="s">
+    </row>
+    <row r="51" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A51" s="6" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="30.75">
-      <c r="A50" s="6" t="s">
+      <c r="B51" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="10" t="s">
+    </row>
+    <row r="52" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" ht="30.75">
-      <c r="A51" s="6" t="s">
+      <c r="B52" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="10" t="s">
+    </row>
+    <row r="53" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="30.75">
-      <c r="A52" s="6" t="s">
+      <c r="B53" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="10" t="s">
+    </row>
+    <row r="54" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" ht="30.75">
-      <c r="A53" s="6" t="s">
+      <c r="B54" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B53" s="10" t="s">
+    </row>
+    <row r="55" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A55" s="6" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" ht="45.75">
-      <c r="A54" s="6" t="s">
+      <c r="B55" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="10" t="s">
+    </row>
+    <row r="56" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" ht="30.75">
-      <c r="A55" s="6" t="s">
+      <c r="B56" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="10" t="s">
+    </row>
+    <row r="57" spans="1:2" ht="48" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" ht="45.75">
-      <c r="A56" s="6" t="s">
+      <c r="B57" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="14" t="s">
+    </row>
+    <row r="58" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" ht="30.75">
-      <c r="A57" s="6" t="s">
+      <c r="B58" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="14" t="s">
+    </row>
+    <row r="59" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" ht="45.75">
-      <c r="A58" s="6" t="s">
+      <c r="B59" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="B58" s="14" t="s">
+    </row>
+    <row r="60" spans="1:2" ht="32" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" ht="30.75">
-      <c r="A59" s="6" t="s">
+      <c r="B60" s="14" t="s">
         <v>116</v>
-      </c>
-      <c r="B59" s="14" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2384,652 +2409,652 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8916CB2-7716-4BBC-942E-3D07018F48E5}">
   <dimension ref="A1:D80"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1640625" style="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="114" style="18" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="18"/>
+    <col min="3" max="16384" width="9.1640625" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A1" s="17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="23.25">
+    <row r="2" spans="1:4" ht="14" x14ac:dyDescent="0.15">
       <c r="A2" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="19" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="14" x14ac:dyDescent="0.15">
+      <c r="A3" s="18" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="18" t="s">
+      <c r="B3" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="19" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A4" s="18" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="23.25">
-      <c r="A4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="19" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="14" x14ac:dyDescent="0.15">
+      <c r="A5" s="18" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="23.25">
-      <c r="A5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="19" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="18" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="18" t="s">
+      <c r="B6" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="18" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A7" s="18" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="23.25">
-      <c r="A7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="19" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A8" s="18" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="23.25">
-      <c r="A8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="B8" s="19" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A9" s="18" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="23.25">
-      <c r="A9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="19" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A10" s="18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="18" t="s">
+      <c r="B10" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="B10" s="18" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="42" x14ac:dyDescent="0.15">
+      <c r="A11" s="18" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="35.25">
-      <c r="A11" s="18" t="s">
+      <c r="B11" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="B11" s="20" t="s">
+    </row>
+    <row r="12" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A12" s="18" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="23.25">
-      <c r="A12" s="18" t="s">
+      <c r="B12" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="B12" s="20" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="14" x14ac:dyDescent="0.15">
+      <c r="A13" s="18" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="B13" s="19" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="14" x14ac:dyDescent="0.15">
+      <c r="A14" s="18" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B14" s="19" t="s">
+    </row>
+    <row r="15" spans="1:4" ht="42" x14ac:dyDescent="0.15">
+      <c r="A15" s="18" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="35.25">
-      <c r="A15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" spans="1:4" ht="28" x14ac:dyDescent="0.15">
+      <c r="A16" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D15" s="21"/>
-    </row>
-    <row r="16" spans="1:4" ht="35.25">
-      <c r="A16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B16" s="19" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A17" s="18" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>149</v>
       </c>
-      <c r="B17" s="19" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A18" s="18" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="23.25">
-      <c r="A18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>151</v>
       </c>
-      <c r="B18" s="19" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A19" s="18" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="18" t="s">
+      <c r="B19" s="19" t="s">
         <v>153</v>
       </c>
-      <c r="B19" s="19" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A20" s="18" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="23.25">
-      <c r="A20" s="18" t="s">
+      <c r="B20" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B20" s="19" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A21" s="18" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="23.25">
-      <c r="A21" s="18" t="s">
+      <c r="B21" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="B21" s="19" t="s">
+    </row>
+    <row r="22" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A22" s="18" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="35.25">
-      <c r="A22" s="18" t="s">
+      <c r="B22" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="B22" s="19" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A23" s="18" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="23.25">
-      <c r="A23" s="18" t="s">
+      <c r="B23" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="B23" s="19" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A24" s="18" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="36.75">
-      <c r="A24" s="18" t="s">
+      <c r="B24" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="B24" s="19" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A25" s="18" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" ht="25.5">
-      <c r="A25" s="18" t="s">
+      <c r="B25" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="B25" s="20" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A26" s="18" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" ht="23.25">
-      <c r="A26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="B26" s="19" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A27" s="18" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" ht="23.25">
-      <c r="A27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="19" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A28" s="18" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" ht="23.25">
-      <c r="A28" s="18" t="s">
+      <c r="B28" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="B28" s="19" t="s">
+    </row>
+    <row r="29" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A29" s="18" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" ht="23.25">
-      <c r="A29" s="18" t="s">
+      <c r="B29" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="B29" s="19" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A30" s="22" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" ht="23.25">
-      <c r="A30" s="22" t="s">
+      <c r="B30" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="B30" s="20" t="s">
+    </row>
+    <row r="31" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A31" s="18" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" ht="23.25">
-      <c r="A31" s="18" t="s">
+      <c r="B31" s="19" t="s">
         <v>177</v>
       </c>
-      <c r="B31" s="19" t="s">
+    </row>
+    <row r="32" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A32" s="18" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" ht="35.25">
-      <c r="A32" s="18" t="s">
+      <c r="B32" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="B32" s="19" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A33" s="18" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" ht="23.25">
-      <c r="A33" s="18" t="s">
+      <c r="B33" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="B33" s="19" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A34" s="18" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" ht="35.25">
-      <c r="A34" s="18" t="s">
+      <c r="B34" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="B34" s="19" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A35" s="18" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" ht="23.25">
-      <c r="A35" s="18" t="s">
+      <c r="B35" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="B35" s="19" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A36" s="18" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" ht="35.25">
-      <c r="A36" s="18" t="s">
+      <c r="B36" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="B36" s="19" t="s">
+    </row>
+    <row r="37" spans="1:2" s="23" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+      <c r="A37" s="23" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" s="23" customFormat="1" ht="23.25">
-      <c r="A37" s="23" t="s">
+      <c r="B37" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="B37" s="24" t="s">
+    </row>
+    <row r="38" spans="1:2" s="23" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="23" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" s="23" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A38" s="23" t="s">
+      <c r="B38" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="B38" s="24" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A39" s="18" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" ht="23.25">
-      <c r="A39" s="18" t="s">
+      <c r="B39" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="B39" s="19" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A40" s="18" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="18" t="s">
+      <c r="B40" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="B40" s="19" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A41" s="18" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" s="18" t="s">
+      <c r="B41" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B41" s="19" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A42" s="18" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" ht="23.25">
-      <c r="A42" s="18" t="s">
+      <c r="B42" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="B42" s="19" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A43" s="18" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" ht="23.25">
-      <c r="A43" s="18" t="s">
+      <c r="B43" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="B43" s="19" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A44" s="18" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
-      <c r="A44" s="18" t="s">
+      <c r="B44" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="B44" s="19" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A45" s="18" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" ht="35.25">
-      <c r="A45" s="18" t="s">
+      <c r="B45" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="B45" s="19" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A46" s="18" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" ht="23.25">
-      <c r="A46" s="18" t="s">
+      <c r="B46" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="B46" s="19" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A47" s="18" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
-      <c r="A47" s="18" t="s">
+      <c r="B47" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="B47" s="19" t="s">
+    </row>
+    <row r="48" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A48" s="18" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" ht="23.25">
-      <c r="A48" s="18" t="s">
+      <c r="B48" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="B48" s="19" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A49" s="18" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="23.25">
-      <c r="A49" s="18" t="s">
+      <c r="B49" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="B49" s="19" t="s">
+    </row>
+    <row r="50" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A50" s="18" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="35.25">
-      <c r="A50" s="18" t="s">
+      <c r="B50" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="B50" s="19" t="s">
+    </row>
+    <row r="51" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A51" s="18" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" ht="23.25">
-      <c r="A51" s="18" t="s">
+      <c r="B51" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="B51" s="19" t="s">
+    </row>
+    <row r="52" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A52" s="18" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="23.25">
-      <c r="A52" s="18" t="s">
+      <c r="B52" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="B52" s="19" t="s">
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A53" s="18" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" s="18" t="s">
+      <c r="B53" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="B53" s="18" t="s">
+    </row>
+    <row r="54" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A54" s="18" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" ht="35.25">
-      <c r="A54" s="18" t="s">
+      <c r="B54" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="B54" s="19" t="s">
+    </row>
+    <row r="55" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A55" s="18" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" ht="23.25">
-      <c r="A55" s="18" t="s">
+      <c r="B55" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="B55" s="19" t="s">
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A56" s="18" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="A56" s="18" t="s">
+      <c r="B56" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="B56" s="18" t="s">
+    </row>
+    <row r="57" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A57" s="18" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" ht="23.25">
-      <c r="A57" s="18" t="s">
+      <c r="B57" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="B57" s="19" t="s">
+    </row>
+    <row r="58" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A58" s="18" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" ht="23.25">
-      <c r="A58" s="18" t="s">
+      <c r="B58" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="B58" s="19" t="s">
+    </row>
+    <row r="59" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A59" s="18" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" s="18" t="s">
+      <c r="B59" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="B59" s="19" t="s">
+    </row>
+    <row r="60" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A60" s="18" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" ht="23.25">
-      <c r="A60" s="18" t="s">
+      <c r="B60" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="B60" s="19" t="s">
+    </row>
+    <row r="61" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A61" s="18" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" ht="23.25">
-      <c r="A61" s="18" t="s">
+      <c r="B61" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="B61" s="19" t="s">
+    </row>
+    <row r="62" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A62" s="18" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" ht="23.25">
-      <c r="A62" s="18" t="s">
+      <c r="B62" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="B62" s="19" t="s">
+    </row>
+    <row r="63" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A63" s="18" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" ht="35.25">
-      <c r="A63" s="18" t="s">
+      <c r="B63" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="B63" s="19" t="s">
+    </row>
+    <row r="64" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A64" s="18" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" ht="23.25">
-      <c r="A64" s="18" t="s">
+      <c r="B64" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="B64" s="19" t="s">
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A65" s="18" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="65" spans="1:2">
-      <c r="A65" s="18" t="s">
+      <c r="B65" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="B65" s="18" t="s">
+    </row>
+    <row r="66" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A66" s="18" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="66" spans="1:2">
-      <c r="A66" s="18" t="s">
+      <c r="B66" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="B66" s="19" t="s">
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A67" s="18" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="67" spans="1:2">
-      <c r="A67" s="18" t="s">
+      <c r="B67" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="B67" s="18" t="s">
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A68" s="18" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="18" t="s">
+      <c r="B68" s="18" t="s">
         <v>251</v>
       </c>
-      <c r="B68" s="18" t="s">
+    </row>
+    <row r="69" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A69" s="18" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" ht="35.25">
-      <c r="A69" s="18" t="s">
+      <c r="B69" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="B69" s="19" t="s">
+    </row>
+    <row r="70" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A70" s="18" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" ht="23.25">
-      <c r="A70" s="18" t="s">
+      <c r="B70" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="B70" s="19" t="s">
+    </row>
+    <row r="71" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A71" s="18" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" ht="46.5">
-      <c r="A71" s="18" t="s">
+      <c r="B71" s="19" t="s">
         <v>257</v>
       </c>
-      <c r="B71" s="19" t="s">
+    </row>
+    <row r="72" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A72" s="18" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" ht="23.25">
-      <c r="A72" s="18" t="s">
+      <c r="B72" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="B72" s="19" t="s">
+    </row>
+    <row r="73" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A73" s="18" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="73" spans="1:2">
-      <c r="A73" s="18" t="s">
+      <c r="B73" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="B73" s="19" t="s">
+    </row>
+    <row r="74" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A74" s="18" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" ht="23.25">
-      <c r="A74" s="18" t="s">
+      <c r="B74" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="B74" s="19" t="s">
+    </row>
+    <row r="75" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A75" s="18" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="75" spans="1:2">
-      <c r="A75" s="18" t="s">
+      <c r="B75" s="19" t="s">
         <v>265</v>
       </c>
-      <c r="B75" s="19" t="s">
+    </row>
+    <row r="76" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A76" s="18" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="18" t="s">
+      <c r="B76" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="B76" s="19" t="s">
+    </row>
+    <row r="77" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A77" s="18" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" ht="23.25">
-      <c r="A77" s="18" t="s">
+      <c r="B77" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="B77" s="19" t="s">
+    </row>
+    <row r="78" spans="1:2" ht="28" x14ac:dyDescent="0.15">
+      <c r="A78" s="18" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="78" spans="1:2" ht="23.25">
-      <c r="A78" s="18" t="s">
+      <c r="B78" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="B78" s="19" t="s">
+    </row>
+    <row r="79" spans="1:2" ht="14" x14ac:dyDescent="0.15">
+      <c r="A79" s="18" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="79" spans="1:2">
-      <c r="A79" s="18" t="s">
+      <c r="B79" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="B79" s="19" t="s">
+    </row>
+    <row r="80" spans="1:2" ht="42" x14ac:dyDescent="0.15">
+      <c r="A80" s="18" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="80" spans="1:2" ht="35.25">
-      <c r="A80" s="18" t="s">
+      <c r="B80" s="19" t="s">
         <v>275</v>
-      </c>
-      <c r="B80" s="19" t="s">
-        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -3040,498 +3065,498 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CACC83A9-B8FE-4EAB-B2A4-3113B263B28E}">
   <dimension ref="A1:B61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="102.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="102.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="21.75">
+    <row r="2" spans="1:2" ht="27" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="21.75">
-      <c r="A3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="B3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="B4" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="B5" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B5" s="3" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
+      <c r="B6" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
+      <c r="B7" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
+      <c r="B8" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="B8" s="3" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
+      <c r="B9" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="B9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="21.75">
-      <c r="A10" t="s">
+      <c r="B10" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="B10" s="3" t="s">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+      <c r="B11" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="B11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
+      <c r="B12" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="B12" s="3" t="s">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+      <c r="B13" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="B13" s="3" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="21.75">
-      <c r="A14" t="s">
+      <c r="B14" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="B14" s="3" t="s">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
+      <c r="B15" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="B15" s="3" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="21.75">
-      <c r="A16" t="s">
+      <c r="B16" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B16" s="3" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="21.75">
-      <c r="A17" t="s">
+      <c r="B17" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="B17" s="3" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="21.75">
-      <c r="A18" t="s">
+      <c r="B18" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="B18" s="3" t="s">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
+      <c r="B19" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="B19" s="3" t="s">
+    </row>
+    <row r="20" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="21.75">
-      <c r="A20" t="s">
+      <c r="B20" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="B20" s="3" t="s">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
+      <c r="B21" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="B21" s="3" t="s">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
+      <c r="B22" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="B22" s="2" t="s">
+    </row>
+    <row r="23" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="21.75">
-      <c r="A23" t="s">
+      <c r="B23" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="B23" s="3" t="s">
+    </row>
+    <row r="24" spans="1:2" ht="40" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="32.25">
-      <c r="A24" t="s">
+      <c r="B24" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="B24" s="3" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" ht="21.75">
-      <c r="A25" t="s">
+      <c r="B25" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="B25" s="3" t="s">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" t="s">
+      <c r="B26" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="B26" s="3" t="s">
+    </row>
+    <row r="27" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" ht="21.75">
-      <c r="A27" t="s">
+      <c r="B27" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="B27" s="3" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="53" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" ht="43.5">
-      <c r="A28" t="s">
+      <c r="B28" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B28" s="3" t="s">
+    </row>
+    <row r="29" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" ht="21.75">
-      <c r="A29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="B29" s="5" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="40" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" ht="32.25">
-      <c r="A30" t="s">
+      <c r="B30" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="B30" s="3" t="s">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" ht="21.75">
-      <c r="A31" t="s">
+      <c r="B31" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="B31" s="3" t="s">
+    </row>
+    <row r="32" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" ht="21.75">
-      <c r="A32" s="6" t="s">
+      <c r="B32" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="B32" s="5" t="s">
+    </row>
+    <row r="33" spans="1:2" ht="53" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" ht="43.5">
-      <c r="A33" t="s">
+      <c r="B33" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="B33" s="3" t="s">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" t="s">
+      <c r="B34" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="B34" s="3" t="s">
+    </row>
+    <row r="35" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" ht="21.75">
-      <c r="A35" t="s">
+      <c r="B35" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="B35" s="3" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" ht="21.75">
-      <c r="A36" t="s">
+      <c r="B36" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="B36" s="3" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" t="s">
+      <c r="B37" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="B37" s="4" t="s">
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="6" t="s">
+      <c r="B38" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="B38" s="5" t="s">
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" t="s">
+      <c r="B39" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="B39" s="3" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" ht="21.75">
-      <c r="A40" t="s">
+      <c r="B40" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="B40" s="3" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" ht="21.75">
-      <c r="A41" t="s">
+      <c r="B41" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="B41" s="3" t="s">
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
-      <c r="A42" t="s">
+      <c r="B42" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="B42" s="3" t="s">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="43" spans="1:2">
-      <c r="A43" t="s">
+      <c r="B43" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="B43" s="3" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="53" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" ht="43.5">
-      <c r="A44" s="6" t="s">
+      <c r="B44" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="B44" s="5" t="s">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
-      <c r="A45" t="s">
+      <c r="B45" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="B45" s="3" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" ht="21.75">
-      <c r="A46" t="s">
+      <c r="B46" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="B46" s="3" t="s">
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="47" spans="1:2">
-      <c r="A47" t="s">
+      <c r="B47" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="B47" s="3" t="s">
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="48" spans="1:2">
-      <c r="A48" t="s">
+      <c r="B48" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="B48" s="3" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="21.75">
-      <c r="A49" t="s">
+      <c r="B49" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="B49" s="3" t="s">
+    </row>
+    <row r="50" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="21.75">
-      <c r="A50" t="s">
+      <c r="B50" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="B50" s="3" t="s">
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
+      <c r="B51" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="B51" s="3" t="s">
+    </row>
+    <row r="52" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="21.75">
-      <c r="A52" t="s">
+      <c r="B52" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="B52" s="3" t="s">
+    </row>
+    <row r="53" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" ht="21.75">
-      <c r="A53" t="s">
+      <c r="B53" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="B53" s="3" t="s">
+    </row>
+    <row r="54" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" ht="21.75">
-      <c r="A54" t="s">
+      <c r="B54" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="B54" s="3" t="s">
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
+      <c r="B55" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="B55" s="3" t="s">
+    </row>
+    <row r="56" spans="1:2" ht="27" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" ht="21.75">
-      <c r="A56" t="s">
+      <c r="B56" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="B56" s="3" t="s">
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" s="6" t="s">
+      <c r="B57" s="15" t="s">
         <v>387</v>
       </c>
-      <c r="B57" s="15" t="s">
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
+      <c r="B58" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="B58" s="3" t="s">
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
+      <c r="B59" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="B59" s="3" t="s">
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" s="6" t="s">
+      <c r="B60" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="B60" s="5" t="s">
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="61" spans="1:2">
-      <c r="A61" t="s">
+      <c r="B61" s="2" t="s">
         <v>395</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -3542,13 +3567,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB257D0D-5074-45A8-B0C8-C14C3BC554BA}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="89.5703125" customWidth="1"/>
+    <col min="2" max="2" width="89.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3556,148 +3581,148 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="42">
+    <row r="2" spans="1:2" ht="31" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>396</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="B2" s="7" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="46" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="42">
-      <c r="A3" t="s">
+      <c r="B3" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="B3" s="7" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="28.5">
-      <c r="A4" t="s">
+      <c r="B4" s="7" t="s">
         <v>401</v>
       </c>
-      <c r="B4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="28.5">
-      <c r="A5" t="s">
+      <c r="B5" s="7" t="s">
         <v>403</v>
       </c>
-      <c r="B5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="42">
-      <c r="A6" t="s">
+      <c r="B6" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="B6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="28.5">
-      <c r="A7" t="s">
+      <c r="B7" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="B7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="28.5">
-      <c r="A8" t="s">
+      <c r="B8" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="B8" s="7" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="28.5">
-      <c r="A9" t="s">
+      <c r="B9" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="B9" s="7" t="s">
+    </row>
+    <row r="10" spans="1:2" ht="46" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="42">
-      <c r="A10" t="s">
+      <c r="B10" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="B10" s="7" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="28.5">
-      <c r="A11" t="s">
+      <c r="B11" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="B11" s="7" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="46" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="56.25">
-      <c r="A12" t="s">
+      <c r="B12" s="7" t="s">
         <v>417</v>
       </c>
-      <c r="B12" s="7" t="s">
+    </row>
+    <row r="13" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="42">
-      <c r="A13" t="s">
+      <c r="B13" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="B13" s="7" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="28.5">
-      <c r="A14" t="s">
+      <c r="B14" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="B14" s="7" t="s">
+    </row>
+    <row r="15" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="28.5">
-      <c r="A15" t="s">
+      <c r="B15" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="B15" s="7" t="s">
+    </row>
+    <row r="16" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="28.5">
-      <c r="A16" s="9" t="s">
+      <c r="B16" s="8" t="s">
         <v>425</v>
       </c>
-      <c r="B16" s="8" t="s">
+    </row>
+    <row r="17" spans="1:2" ht="31" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="28.5">
-      <c r="A17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="B17" s="8" t="s">
+    </row>
+    <row r="18" spans="1:2" ht="46" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="42">
-      <c r="A18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>429</v>
       </c>
-      <c r="B18" s="8" t="s">
+    </row>
+    <row r="19" spans="1:2" ht="46" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="42">
-      <c r="A19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>431</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>